<commit_message>
update Penyulh Password setting
</commit_message>
<xml_diff>
--- a/public/data_padi/data_padi.xlsx
+++ b/public/data_padi/data_padi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/USER/Documents/PHP Project/SINTREN/public/data_padi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E585E96A-6D56-4840-ABF9-07F5A6C5A899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3536719-F570-0744-9E34-E1C876076DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4180" yWindow="500" windowWidth="26220" windowHeight="20500" firstSheet="5" activeTab="6" xr2:uid="{43C780A0-AB2E-2C45-B813-93E326D04524}"/>
+    <workbookView xWindow="4180" yWindow="500" windowWidth="26220" windowHeight="20500" activeTab="5" xr2:uid="{43C780A0-AB2E-2C45-B813-93E326D04524}"/>
   </bookViews>
   <sheets>
     <sheet name="tahun2010" sheetId="1" r:id="rId1"/>
@@ -1539,6 +1539,14 @@
       <c r="P32" s="2"/>
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="E33">
+        <f>SUM(E2:E32)</f>
+        <v>239788</v>
+      </c>
+      <c r="F33">
+        <f>SUM(F2:F32)</f>
+        <v>239698</v>
+      </c>
       <c r="K33" s="8"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -4021,7 +4029,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C02CFB4-1D2F-0D4A-80A1-5D1C5E64495A}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -4758,6 +4766,12 @@
       </c>
       <c r="G32" s="11">
         <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.2">
+      <c r="G33">
+        <f>SUM(G2:G32)</f>
+        <v>4078</v>
       </c>
     </row>
   </sheetData>
@@ -7005,7 +7019,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A252966D-FF78-994D-9BEE-146F581DA76D}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -7742,6 +7756,12 @@
       </c>
       <c r="G32" s="11">
         <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.2">
+      <c r="G33">
+        <f>SUM(G2:G32)</f>
+        <v>21463</v>
       </c>
     </row>
   </sheetData>

</xml_diff>